<commit_message>
feat: land shop stage, dig equipment effects, and warrior appearance packs
Ship Mode2 shop runtime, Elctr/explosives dig systems, equipment UI assets, and App_1-3 warrior appearance/prefab content with matching SPEC updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/主角_装备配置表_Protagonist_ProtagonistEquipmentConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/主角_装备配置表_Protagonist_ProtagonistEquipmentConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -996,7 +996,6 @@
           <t>Icon_MinerLamp</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>1</t>
@@ -1015,6 +1014,237 @@
       <c r="I13" t="inlineStr">
         <is>
           <t>每级增加Q4/Q5/Q6生成权重10（满级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Equip_Detector</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>探测器</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Icon_Detector</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>DigProcessSpawnCountBonus_1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>每级增加过程生成坟墓数量+1（1级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Equip_Detector</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>探测器</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Icon_Detector</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>DigProcessSpawnCountBonus_2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>每级增加过程生成坟墓数量+1（2级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Equip_Detector</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>探测器</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Icon_Detector</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>DigProcessSpawnCountBonus_3</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>每级增加过程生成坟墓数量+1（3级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Equip_Detector</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>探测器</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Icon_Detector</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>DigProcessSpawnCountBonus_4</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>每级增加过程生成坟墓数量+1（4级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Equip_Detector</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>探测器</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Icon_Detector</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>DigProcessSpawnCountBonus_5</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>每级增加过程生成坟墓数量+1（满级）</t>
         </is>
       </c>
     </row>

</xml_diff>